<commit_message>
Fix what a first-time reader could not follow on the site
</commit_message>
<xml_diff>
--- a/model/domain_valuation_model.xlsx
+++ b/model/domain_valuation_model.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{30FC6DAC-C175-4B57-A986-50D8F4B7C680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE4CF33B-C050-498B-BF75-B1FF641A9E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -462,7 +462,7 @@
     <t>30 May 2025</t>
   </si>
   <si>
-    <t>10-year Commonwealth Government bond yield. On 5 October 2026 I chose this over the expert's 4.3% (and over 4.366%, the RBA yield at 31 December 2024) so that the 0.05 point difference shows as its own step in the gap bridge.</t>
+    <t>10-year Commonwealth Government bond yield. On 5 October 2026 I chose this over the expert's 4.3% (and over 4.366%, the RBA yield at 31 December 2024). My DCF uses the expert's adopted discount rate range, so the 0.05 point difference does not change my value (docs/BASE_CASE.md, discount rate).</t>
   </si>
   <si>
     <t>expert_risk_free_rate_pct</t>

</xml_diff>